<commit_message>
100%: more benchmarks: * overall WAPE * group WAPE * custom APE
</commit_message>
<xml_diff>
--- a/predictions/ARIMA.xlsx
+++ b/predictions/ARIMA.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I22"/>
+  <dimension ref="A1:L22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -462,6 +462,21 @@
           <t>order</t>
         </is>
       </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>custom_ape</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>group_wape</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>wape</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -499,6 +514,15 @@
           <t>(1, 1, 1)</t>
         </is>
       </c>
+      <c r="J2" t="n">
+        <v>1.562</v>
+      </c>
+      <c r="K2" t="n">
+        <v>2.355</v>
+      </c>
+      <c r="L2" t="n">
+        <v>2.253</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -536,6 +560,15 @@
           <t>(0, 1, 2)</t>
         </is>
       </c>
+      <c r="J3" t="n">
+        <v>1.563</v>
+      </c>
+      <c r="K3" t="n">
+        <v>5.165</v>
+      </c>
+      <c r="L3" t="n">
+        <v>2.253</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -573,6 +606,15 @@
           <t>(0, 1, 2)</t>
         </is>
       </c>
+      <c r="J4" t="n">
+        <v>0.133</v>
+      </c>
+      <c r="K4" t="n">
+        <v>0.959</v>
+      </c>
+      <c r="L4" t="n">
+        <v>2.253</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -608,6 +650,15 @@
           <t>(2, 1, 0)</t>
         </is>
       </c>
+      <c r="J5" t="n">
+        <v>0.022</v>
+      </c>
+      <c r="K5" t="n">
+        <v>0.993</v>
+      </c>
+      <c r="L5" t="n">
+        <v>2.253</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -643,6 +694,15 @@
           <t>(0, 1, 2)</t>
         </is>
       </c>
+      <c r="J6" t="n">
+        <v>26.206</v>
+      </c>
+      <c r="K6" t="n">
+        <v>46.191</v>
+      </c>
+      <c r="L6" t="n">
+        <v>2.253</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -678,6 +738,15 @@
           <t>(2, 1, 0)</t>
         </is>
       </c>
+      <c r="J7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K7" t="n">
+        <v>1</v>
+      </c>
+      <c r="L7" t="n">
+        <v>2.253</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -713,6 +782,15 @@
           <t>(0, 0, 0)</t>
         </is>
       </c>
+      <c r="J8" t="n">
+        <v>0.092</v>
+      </c>
+      <c r="K8" t="n">
+        <v>1.083</v>
+      </c>
+      <c r="L8" t="n">
+        <v>2.253</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -750,6 +828,15 @@
           <t>(0, 1, 2)</t>
         </is>
       </c>
+      <c r="J9" t="n">
+        <v>0.535</v>
+      </c>
+      <c r="K9" t="n">
+        <v>2.355</v>
+      </c>
+      <c r="L9" t="n">
+        <v>2.253</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -785,6 +872,15 @@
           <t>(0, 1, 2)</t>
         </is>
       </c>
+      <c r="J10" t="n">
+        <v>2.042</v>
+      </c>
+      <c r="K10" t="n">
+        <v>5.165</v>
+      </c>
+      <c r="L10" t="n">
+        <v>2.253</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -820,6 +916,15 @@
           <t>(0, 1, 2)</t>
         </is>
       </c>
+      <c r="J11" t="n">
+        <v>0.78</v>
+      </c>
+      <c r="K11" t="n">
+        <v>0.959</v>
+      </c>
+      <c r="L11" t="n">
+        <v>2.253</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -857,6 +962,15 @@
           <t>(2, 1, 0)</t>
         </is>
       </c>
+      <c r="J12" t="n">
+        <v>0.304</v>
+      </c>
+      <c r="K12" t="n">
+        <v>0.993</v>
+      </c>
+      <c r="L12" t="n">
+        <v>2.253</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -892,6 +1006,15 @@
           <t>(0, 1, 2)</t>
         </is>
       </c>
+      <c r="J13" t="n">
+        <v>14.958</v>
+      </c>
+      <c r="K13" t="n">
+        <v>46.191</v>
+      </c>
+      <c r="L13" t="n">
+        <v>2.253</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -927,6 +1050,15 @@
           <t>(2, 1, 0)</t>
         </is>
       </c>
+      <c r="J14" t="n">
+        <v>0</v>
+      </c>
+      <c r="K14" t="n">
+        <v>1</v>
+      </c>
+      <c r="L14" t="n">
+        <v>2.253</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -964,6 +1096,15 @@
           <t>(0, 1, 2)</t>
         </is>
       </c>
+      <c r="J15" t="n">
+        <v>0.041</v>
+      </c>
+      <c r="K15" t="n">
+        <v>1.083</v>
+      </c>
+      <c r="L15" t="n">
+        <v>2.253</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1001,6 +1142,15 @@
           <t>(0, 1, 1)</t>
         </is>
       </c>
+      <c r="J16" t="n">
+        <v>0.258</v>
+      </c>
+      <c r="K16" t="n">
+        <v>2.355</v>
+      </c>
+      <c r="L16" t="n">
+        <v>2.253</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1038,6 +1188,15 @@
           <t>(0, 1, 1)</t>
         </is>
       </c>
+      <c r="J17" t="n">
+        <v>1.56</v>
+      </c>
+      <c r="K17" t="n">
+        <v>5.165</v>
+      </c>
+      <c r="L17" t="n">
+        <v>2.253</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1075,6 +1234,15 @@
           <t>(0, 1, 1)</t>
         </is>
       </c>
+      <c r="J18" t="n">
+        <v>0.047</v>
+      </c>
+      <c r="K18" t="n">
+        <v>0.959</v>
+      </c>
+      <c r="L18" t="n">
+        <v>2.253</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1112,6 +1280,15 @@
           <t>(1, 0, 0)</t>
         </is>
       </c>
+      <c r="J19" t="n">
+        <v>0.667</v>
+      </c>
+      <c r="K19" t="n">
+        <v>0.993</v>
+      </c>
+      <c r="L19" t="n">
+        <v>2.253</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1149,6 +1326,15 @@
           <t>(0, 1, 2)</t>
         </is>
       </c>
+      <c r="J20" t="n">
+        <v>5.027</v>
+      </c>
+      <c r="K20" t="n">
+        <v>46.191</v>
+      </c>
+      <c r="L20" t="n">
+        <v>2.253</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1186,6 +1372,15 @@
           <t>(2, 1, 0)</t>
         </is>
       </c>
+      <c r="J21" t="n">
+        <v>1</v>
+      </c>
+      <c r="K21" t="n">
+        <v>1</v>
+      </c>
+      <c r="L21" t="n">
+        <v>2.253</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1222,6 +1417,15 @@
         <is>
           <t>(1, 0, 1)</t>
         </is>
+      </c>
+      <c r="J22" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="K22" t="n">
+        <v>1.083</v>
+      </c>
+      <c r="L22" t="n">
+        <v>2.253</v>
       </c>
     </row>
   </sheetData>

</xml_diff>